<commit_message>
update output excel file
</commit_message>
<xml_diff>
--- a/Output_file.xlsx
+++ b/Output_file.xlsx
@@ -3,10 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="John Doe - Input" sheetId="1" r:id="rId1"/>
-    <sheet name="John Doe - Output" sheetId="2" r:id="rId2"/>
-    <sheet name="Peter Parker - Input" sheetId="3" r:id="rId3"/>
-    <sheet name="Peter Parker - Output" sheetId="4" r:id="rId4"/>
+    <sheet name="Alice Nguyen - Input" sheetId="1" r:id="rId1"/>
+    <sheet name="Alice Nguyen - Output" sheetId="2" r:id="rId2"/>
+    <sheet name="Edna Kowalski - Input" sheetId="3" r:id="rId3"/>
+    <sheet name="Edna Kowalski - Output" sheetId="4" r:id="rId4"/>
+    <sheet name="Robert Singh - Input" sheetId="5" r:id="rId5"/>
+    <sheet name="Robert Singh - Output" sheetId="6" r:id="rId6"/>
+    <sheet name="Thomas Brennan - Input" sheetId="7" r:id="rId7"/>
+    <sheet name="Thomas Brennan - Output" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
@@ -204,18 +208,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE8F5E9"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8F5E9"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFF2DCDB"/>
         <bgColor/>
       </patternFill>
@@ -235,6 +227,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF8E1"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F5E9"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F5E9"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -881,7 +885,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -891,7 +895,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="3" t="str">
-        <v>Progress Notes — John Doe</v>
+        <v>Progress Notes — Alice Nguyen</v>
       </c>
       <c r="B1" s="4" t="str">
         <v/>
@@ -905,7 +909,7 @@
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="5" t="str">
-        <v>2 consecutive daily progress notes uploaded for compliance checking.</v>
+        <v>3 consecutive daily progress notes uploaded for compliance checking.</v>
       </c>
       <c r="B2" s="6" t="str">
         <v/>
@@ -936,24 +940,21 @@
         <v>Day 1</v>
       </c>
       <c r="B4" s="10" t="str">
-        <v>2026-06-17</v>
+        <v>10 June 2025</v>
       </c>
       <c r="C4" s="11" t="str">
         <v>Uploaded</v>
       </c>
       <c r="D4" s="12" t="str" xml:space="preserve">
-        <v xml:space="preserve">"Progress Note — Fall Incident
-Resident: Thomas Brennan  |  Room: 9F  |  DOB: 22/05/1941
-Date: 10 June 2025  |  Time of fall: 13:55
-Resident witnessed falling in the activity room. Complaining of left knee pain — rates 5/10. No visible injury. Alert and orientated. Able to move all limbs.
-Immediate actions: Assisted to chair. Comfort measures applied. Call bell within reach.
-Vital signs: BP 145/88, HR 82, RR 16, Temp 36.6, SpO2 97%.
-GP (Dr Maria Santos) notified at 14:15. Advised to monitor and reassess tomorrow.
-NOK: Wife (Catherine Brennan) notified at 14:30. Acknowledged, will visit this evening.
-Risk factors: Two previous falls this year. On Warfarin — bleeding risk noted. Uses walking stick.
-Walking stick was in reach at time of fall.
-Care plan reviewed and updated: Yes. Walking stick protocol reinforced. Falls risk score reassessed — HIGH."
-</v>
+        <v xml:space="preserve">Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Complaining of lower back pain — rates 4/10. No visible injury. Alert and orientated. Able to move all limbs.
+Immediate actions: Assisted back to bed. Comfort position established. Call bell placed within reach.
+GP (Dr Fiona Walsh) notified at 08:30. Advised to monitor and keep mobile. No X-ray required at this stage.
+NOK: Son (Michael Nguyen) notified. Acknowledged.
+Risk factors: One previous fall three months ago. On Metformin for diabetes — no anticoagulants. No mobility aid in use.
+Care plan reviewed and updated: Yes. Non-slip footwear added as intervention. Falls risk score reassessed — MEDIUM.</v>
       </c>
     </row>
     <row r="5" ht="80" customHeight="1" xml:space="preserve">
@@ -967,21 +968,29 @@
         <v>Uploaded</v>
       </c>
       <c r="D5" s="12" t="str" xml:space="preserve">
-        <v xml:space="preserve">Progress Note — Day 2 Post-Fall_x000d_
-Resident: John Doe  |  Room: 8B_x000d_
-Date: 11 June 2025_x000d_
-_x000d_
-Pain update: Left knee pain has improved since yesterday — resident rates 2/10 this morning. No new pain reported._x000d_
-_x000d_
-Mobility: Resident able to full weight-bear on both legs without assistance. Walking to bathroom and back independently using walking frame. Gait appears steady._x000d_
-_x000d_
-Vital signs: BP 142/84, HR 76, RR 15, Temp 36.6, SpO2 98%._x000d_
-_x000d_
-No new symptoms since Day 1 — no new bruising, swelling, or behavioural changes observed._x000d_
-_x000d_
-GP follow-up: Contacted Dr Santos at 09:30 to update on pain improvement and weight-bearing status. Dr Santos advised no X-ray required at this stage given improvement. Advised to continue monitoring and reassess if pain worsens._x000d_
-_x000d_
-Care plan: No changes required today. Walking frame placement confirmed in place.</v>
+        <v xml:space="preserve">Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms noted. No further falls overnight.</v>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1" xml:space="preserve">
+      <c r="A6" s="9" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B6" s="10" t="str">
+        <v>12 June 2025</v>
+      </c>
+      <c r="C6" s="11" t="str">
+        <v>Uploaded</v>
+      </c>
+      <c r="D6" s="12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.</v>
       </c>
     </row>
   </sheetData>
@@ -990,14 +999,14 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D14"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1007,7 +1016,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="4" t="str">
-        <v>Checker Output — John Doe</v>
+        <v>Checker Output — Alice Nguyen</v>
       </c>
       <c r="B1" s="4" t="str">
         <v/>
@@ -1021,7 +1030,7 @@
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="6" t="str">
-        <v>All 2 days reviewed against the Falls Management Policy.</v>
+        <v>All 3 days reviewed against the Falls Management Policy.</v>
       </c>
       <c r="B2" s="6" t="str">
         <v/>
@@ -1052,27 +1061,153 @@
         <v>Day 1</v>
       </c>
       <c r="B4" s="14" t="str">
-        <v>✅ Complete</v>
+        <v>🚩 Missing</v>
       </c>
       <c r="C4" s="14" t="str">
-        <v>All fields present</v>
+        <v>Vital signs not recorded</v>
       </c>
       <c r="D4" s="14" t="str">
-        <v>No flags raised</v>
+        <v>Policy requires recording actual values for vital signs (BP, HR, RR, Temperature, SpO2). No vital signs recorded in the note.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="str">
+        <v>Day 1</v>
+      </c>
+      <c r="B5" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C5" s="14" t="str">
+        <v>NOK name and notification time absent</v>
+      </c>
+      <c r="D5" s="14" t="str">
+        <v>Policy requires documenting the NOK's name and exact notification time. Note states 'NOK: Son (Michael Nguyen) notified. Acknowledged.' but does not include the time of notification.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="str">
         <v>Day 2</v>
       </c>
-      <c r="B5" s="14" t="str">
-        <v>✅ Complete</v>
-      </c>
-      <c r="C5" s="14" t="str">
-        <v>All fields present</v>
-      </c>
-      <c r="D5" s="14" t="str">
-        <v>No flags raised</v>
+      <c r="B6" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C6" s="14" t="str">
+        <v>Pain status not updated</v>
+      </c>
+      <c r="D6" s="14" t="str">
+        <v>Policy requires a numeric 0-10 pain score or explicit pain status update. Note states 'Back pain seems a bit better today' but does not include a numeric pain score or clear status update.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B7" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C7" s="14" t="str">
+        <v>GP follow-up not documented</v>
+      </c>
+      <c r="D7" s="14" t="str">
+        <v>Policy requires documentation of GP follow-up or actions taken based on GP advice. No mention of GP follow-up is documented in the note.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B8" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C8" s="14" t="str">
+        <v>Care plan changes not documented</v>
+      </c>
+      <c r="D8" s="14" t="str">
+        <v>Policy requires documentation of care plan changes or a statement that no changes are needed. No mention of care plan changes is documented in the note.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B9" s="16" t="str">
+        <v>⚠️ Vague</v>
+      </c>
+      <c r="C9" s="16" t="str">
+        <v>Mobility status unclear</v>
+      </c>
+      <c r="D9" s="16" t="str">
+        <v>Policy requires explicit confirmation of weight-bearing ability without pain. Note states 'Up and moving around,' which is vague and does not confirm weight-bearing status.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B10" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C10" s="14" t="str">
+        <v>Pain outcome not clinically confirmed</v>
+      </c>
+      <c r="D10" s="14" t="str">
+        <v>Policy requires pain outcome to be clinically confirmed. Note states 'Alice in good spirits' but does not confirm pain status as resolved, ongoing, or with a plan.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B11" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C11" s="14" t="str">
+        <v>Mobility not confirmed at baseline</v>
+      </c>
+      <c r="D11" s="14" t="str">
+        <v>Policy requires mobility to be explicitly confirmed at baseline or documented as reduced with a plan. No mention of mobility, fall status, or physical capability in the note.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B12" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C12" s="14" t="str">
+        <v>Outstanding actions not documented</v>
+      </c>
+      <c r="D12" s="14" t="str">
+        <v>Policy requires documentation of outstanding actions from prior days. No reference to any outstanding actions or their resolution in the note.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B13" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C13" s="14" t="str">
+        <v>Incident not formally closed</v>
+      </c>
+      <c r="D13" s="14" t="str">
+        <v>Policy requires formal closure of incidents. No statement about post-fall monitoring or incident closure in the note.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B14" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C14" s="14" t="str">
+        <v>Falls prevention plan not reviewed</v>
+      </c>
+      <c r="D14" s="14" t="str">
+        <v>Policy requires confirmation that the falls prevention plan was reviewed or discussed. No mention of a falls prevention plan in the note.</v>
       </c>
     </row>
   </sheetData>
@@ -1081,7 +1216,7 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D14"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1098,7 +1233,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="4" t="str">
-        <v>Progress Notes — Peter Parker</v>
+        <v>Progress Notes — Edna Kowalski</v>
       </c>
       <c r="B1" s="4" t="str">
         <v/>
@@ -1149,19 +1284,16 @@
         <v>Uploaded</v>
       </c>
       <c r="D4" s="12" t="str" xml:space="preserve">
-        <v xml:space="preserve">Progress Note — Fall Incident_x000d_
-Resident: Peter Parker  |  Room: 3D_x000d_
-Date: 10 June 2025  |  Time of fall: 14:30_x000d_
-_x000d_
-Resident found on floor in corridor near nurses station. Witnessed by AIN Tom Baxter. Complaining of right hip pain. Alert and orientated. No visible injury._x000d_
-_x000d_
-Immediate actions: Assisted back to wheelchair. Comfort measures applied._x000d_
-_x000d_
-GP (Dr Kevin Park) notified. Advised to monitor._x000d_
-Family has been informed._x000d_
-_x000d_
-Risk factors: History of falls. On blood pressure medication._x000d_
-Care plan: Will update.</v>
+        <v xml:space="preserve">Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of left ankle pain. No visible laceration. Alert and orientated. Able to weight-bear with discomfort.
+Immediate actions: Assisted to chair. Left ankle elevated and ice applied.
+Vital signs: BP 130/78, HR 72, RR 14, Temp 36.3, SpO2 99%.
+GP (Dr Linda Chow) notified at 17:00. Advised to monitor swelling overnight. If unable to weight-bear by morning, arrange X-ray.
+NOK: Husband (Stan Kowalski) notified at 17:10. Acknowledged and stated he will visit tonight.
+Risk factors: First recorded fall. Not on anticoagulants. Walking without aid.
+Care plan reviewed and updated: Yes. Footwear check added as daily intervention.</v>
       </c>
     </row>
     <row r="5" ht="80" customHeight="1" xml:space="preserve">
@@ -1175,11 +1307,13 @@
         <v>Uploaded</v>
       </c>
       <c r="D5" s="12" t="str" xml:space="preserve">
-        <v xml:space="preserve">Progress Note_x000d_
-Resident: Peter Parker  |  Room: 3D_x000d_
-Date: 11 June 2025_x000d_
-_x000d_
-Peter had a quiet night. Seems okay this morning. Ate breakfast.</v>
+        <v xml:space="preserve">Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able to weight-bear on left foot. Walked to dining room for breakfast independently.
+Vitals: BP 128/76, HR 70, RR 14, Temp 36.4, SpO2 99%.
+No new symptoms. No new bruising or swelling beyond the ankle. Husband visited last night as planned.</v>
       </c>
     </row>
     <row r="6" ht="80" customHeight="1" xml:space="preserve">
@@ -1193,11 +1327,13 @@
         <v>Uploaded</v>
       </c>
       <c r="D6" s="12" t="str" xml:space="preserve">
-        <v xml:space="preserve">Progress Note_x000d_
-Resident: Peter Parker  |  Room: 3D_x000d_
-Date: 12 June 2025_x000d_
-_x000d_
-Peter is doing much better. No further falls. Family visited.</v>
+        <v xml:space="preserve">Progress Note — Day 3 Post-Fall Closure
+Resident: Edna Kowalski  |  Room: 2B
+Date: 12 June 2025
+Left ankle pain fully resolved — rates 0/10. Full weight-bearing confirmed, mobilising at baseline without any gait concerns.
+X-ray was not required — resident was able to weight-bear on Day 2 as confirmed above, consistent with GP's conditional advice. No outstanding clinical actions.
+Incident formally closed. Post-fall 72-hour monitoring period complete. No further follow-up required.
+Falls prevention plan reviewed with resident and husband during his visit this evening. Footwear check intervention confirmed in care plan. Both verbally acknowledged the updated plan. Falls risk score documented — LOW.</v>
       </c>
     </row>
   </sheetData>
@@ -1213,7 +1349,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1223,7 +1359,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="4" t="str">
-        <v>Checker Output — Peter Parker</v>
+        <v>Checker Output — Edna Kowalski</v>
       </c>
       <c r="B1" s="4" t="str">
         <v/>
@@ -1264,255 +1400,73 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="str">
+      <c r="A4" s="14" t="str">
         <v>Day 1</v>
       </c>
-      <c r="B4" s="16" t="str">
-        <v>🚩 Missing</v>
-      </c>
-      <c r="C4" s="16" t="str">
+      <c r="B4" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C4" s="14" t="str">
         <v>Pain scale not documented</v>
       </c>
-      <c r="D4" s="16" t="str">
-        <v>Policy requires a numeric pain score (0-10). Note states 'complaining of right hip pain' but does not include a specific pain scale.</v>
+      <c r="D4" s="14" t="str">
+        <v>Policy requires a numeric pain score (0-10) to be documented. Note states 'Resident complains of left ankle pain' but does not include a specific pain score.</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="str">
+      <c r="A5" s="14" t="str">
         <v>Day 1</v>
       </c>
-      <c r="B5" s="16" t="str">
-        <v>🚩 Missing</v>
-      </c>
-      <c r="C5" s="16" t="str">
-        <v>Limb movement not documented</v>
-      </c>
-      <c r="D5" s="16" t="str">
-        <v>Policy requires explicit documentation of limb movement ability. Note states 'assisted back to wheelchair' and 'no visible injury' but does not confirm limb movement.</v>
+      <c r="B5" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C5" s="14" t="str">
+        <v>Falls risk score not reassessed</v>
+      </c>
+      <c r="D5" s="14" t="str">
+        <v>Policy requires a reassessed falls risk score to be documented after a fall. No falls risk score is recorded in the note.</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="str">
-        <v>Day 1</v>
-      </c>
-      <c r="B6" s="16" t="str">
-        <v>🚩 Missing</v>
-      </c>
-      <c r="C6" s="16" t="str">
-        <v>Vital signs not recorded</v>
-      </c>
-      <c r="D6" s="16" t="str">
-        <v>Policy requires vital signs including BP, HR, RR, Temperature, and SpO2 to be recorded. No vital signs are documented.</v>
+      <c r="A6" s="14" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B6" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C6" s="14" t="str">
+        <v>GP follow-up not documented</v>
+      </c>
+      <c r="D6" s="14" t="str">
+        <v>Policy requires documentation of GP follow-up or actions taken based on prior GP advice. No mention of GP review, X-ray arrangement, or monitoring per GP advice is included in the note.</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="str">
-        <v>Day 1</v>
-      </c>
-      <c r="B7" s="16" t="str">
-        <v>🚩 Missing</v>
-      </c>
-      <c r="C7" s="16" t="str">
-        <v>GP notification time not documented</v>
-      </c>
-      <c r="D7" s="16" t="str">
-        <v>Policy requires GP notification time to be documented. Note states 'GP (Dr Kevin Park) notified' but does not include the time of notification.</v>
+      <c r="A7" s="14" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B7" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C7" s="14" t="str">
+        <v>Care plan changes not documented</v>
+      </c>
+      <c r="D7" s="14" t="str">
+        <v>Policy requires documentation of care plan changes or a statement that no changes are needed. The note does not address the care plan at all.</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="str">
-        <v>Day 1</v>
-      </c>
-      <c r="B8" s="16" t="str">
-        <v>🚩 Missing</v>
-      </c>
-      <c r="C8" s="16" t="str">
-        <v>NOK name and notification time absent</v>
-      </c>
-      <c r="D8" s="16" t="str">
-        <v>Policy requires NOK name and notification time to be documented. Note states 'Family has been informed' but does not specify the name or time.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="16" t="str">
-        <v>Day 1</v>
-      </c>
-      <c r="B9" s="16" t="str">
-        <v>🚩 Missing</v>
-      </c>
-      <c r="C9" s="16" t="str">
-        <v>Falls risk score not reassessed</v>
-      </c>
-      <c r="D9" s="16" t="str">
-        <v>Policy requires falls risk score to be reassessed and documented. No falls risk score reassessment is recorded.</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="17" t="str">
-        <v>Day 1</v>
-      </c>
-      <c r="B10" s="18" t="str">
-        <v>⚠️ Vague</v>
-      </c>
-      <c r="C10" s="18" t="str">
-        <v>Care plan update unconfirmed</v>
-      </c>
-      <c r="D10" s="18" t="str">
-        <v>Policy requires confirmation of care plan review and update. Note states 'Care plan: Will update' but does not confirm if the update has been completed.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="16" t="str">
-        <v>Day 2</v>
-      </c>
-      <c r="B11" s="16" t="str">
-        <v>🚩 Missing</v>
-      </c>
-      <c r="C11" s="16" t="str">
-        <v>Pain status not updated</v>
-      </c>
-      <c r="D11" s="16" t="str">
-        <v>Policy requires explicit mention of current pain status or a numeric pain score. No reference to pain or comfort is made in the note.</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="16" t="str">
-        <v>Day 2</v>
-      </c>
-      <c r="B12" s="16" t="str">
-        <v>🚩 Missing</v>
-      </c>
-      <c r="C12" s="16" t="str">
-        <v>New symptoms not assessed</v>
-      </c>
-      <c r="D12" s="16" t="str">
-        <v>Policy requires explicit assessment of new symptoms. No mention of new symptoms or lack thereof is made in the note.</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="str">
-        <v>Day 2</v>
-      </c>
-      <c r="B13" s="16" t="str">
-        <v>🚩 Missing</v>
-      </c>
-      <c r="C13" s="16" t="str">
-        <v>Vital signs not recorded</v>
-      </c>
-      <c r="D13" s="16" t="str">
-        <v>Policy requires a full set of vital signs (BP, HR, RR, Temperature, SpO2). No vital signs are recorded in the note.</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="16" t="str">
-        <v>Day 2</v>
-      </c>
-      <c r="B14" s="16" t="str">
-        <v>🚩 Missing</v>
-      </c>
-      <c r="C14" s="16" t="str">
-        <v>GP follow-up not documented</v>
-      </c>
-      <c r="D14" s="16" t="str">
-        <v>Policy requires documentation of GP follow-up or actions taken based on GP advice. No mention of GP follow-up is made in the note.</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="16" t="str">
-        <v>Day 2</v>
-      </c>
-      <c r="B15" s="16" t="str">
-        <v>🚩 Missing</v>
-      </c>
-      <c r="C15" s="16" t="str">
-        <v>Care plan changes not documented</v>
-      </c>
-      <c r="D15" s="16" t="str">
-        <v>Policy requires documentation of care plan changes or confirmation that there are no changes. No reference to the care plan is made in the note.</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="18" t="str">
-        <v>Day 2</v>
-      </c>
-      <c r="B16" s="18" t="str">
-        <v>⚠️ Vague</v>
-      </c>
-      <c r="C16" s="18" t="str">
-        <v>Mobility status unclear</v>
-      </c>
-      <c r="D16" s="18" t="str">
-        <v>Policy requires explicit confirmation of mobility or weight-bearing status. Note states 'seems okay' and 'ate breakfast,' but these are vague and do not confirm mobility or weight-bearing ability.</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="16" t="str">
+      <c r="A8" s="17" t="str">
         <v>Day 3</v>
       </c>
-      <c r="B17" s="16" t="str">
-        <v>🚩 Missing</v>
-      </c>
-      <c r="C17" s="16" t="str">
-        <v>Outstanding actions not documented</v>
-      </c>
-      <c r="D17" s="16" t="str">
-        <v>Policy requires documentation of outstanding actions from prior days. No mention of outstanding actions is present in the note.</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="str">
-        <v>Day 3</v>
-      </c>
-      <c r="B18" s="16" t="str">
-        <v>🚩 Missing</v>
-      </c>
-      <c r="C18" s="16" t="str">
-        <v>Incident not formally closed</v>
-      </c>
-      <c r="D18" s="16" t="str">
-        <v>Policy requires a formal statement that the post-fall monitoring period is complete and the incident is closed. No such statement is included in the note.</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="str">
-        <v>Day 3</v>
-      </c>
-      <c r="B19" s="16" t="str">
-        <v>🚩 Missing</v>
-      </c>
-      <c r="C19" s="16" t="str">
-        <v>Falls prevention plan not reviewed</v>
-      </c>
-      <c r="D19" s="16" t="str">
-        <v>Policy requires confirmation that the updated falls prevention plan was reviewed or discussed with the resident and/or family. No mention of a falls prevention plan review is present in the note.</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="18" t="str">
-        <v>Day 3</v>
-      </c>
-      <c r="B20" s="18" t="str">
-        <v>⚠️ Vague</v>
-      </c>
-      <c r="C20" s="18" t="str">
-        <v>Pain outcome not clinically confirmed</v>
-      </c>
-      <c r="D20" s="18" t="str">
-        <v>Policy requires pain outcome to be clinically confirmed. Note states 'doing much better,' but this is vague and not a clinical confirmation of pain resolution or ongoing status.</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="18" t="str">
-        <v>Day 3</v>
-      </c>
-      <c r="B21" s="18" t="str">
-        <v>⚠️ Vague</v>
-      </c>
-      <c r="C21" s="18" t="str">
-        <v>Mobility not confirmed at baseline</v>
-      </c>
-      <c r="D21" s="18" t="str">
-        <v>Policy requires mobility to be explicitly confirmed as returned to baseline or documented as reduced with a follow-up plan. Note states 'no further falls,' but this does not confirm baseline mobility status.</v>
+      <c r="B8" s="18" t="str">
+        <v>✅ Complete</v>
+      </c>
+      <c r="C8" s="18" t="str">
+        <v>All fields present</v>
+      </c>
+      <c r="D8" s="18" t="str">
+        <v>No flags raised</v>
       </c>
     </row>
   </sheetData>
@@ -1521,7 +1475,658 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D6"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="90.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="4" t="str">
+        <v>Progress Notes — Robert Singh</v>
+      </c>
+      <c r="B1" s="4" t="str">
+        <v/>
+      </c>
+      <c r="C1" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D1" s="4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="6" t="str">
+        <v>3 consecutive daily progress notes uploaded for compliance checking.</v>
+      </c>
+      <c r="B2" s="6" t="str">
+        <v/>
+      </c>
+      <c r="C2" s="6" t="str">
+        <v/>
+      </c>
+      <c r="D2" s="6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="8" t="str">
+        <v>Day</v>
+      </c>
+      <c r="B3" s="8" t="str">
+        <v>Date</v>
+      </c>
+      <c r="C3" s="8" t="str">
+        <v>Source</v>
+      </c>
+      <c r="D3" s="8" t="str">
+        <v>Progress Note</v>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1" xml:space="preserve">
+      <c r="A4" s="9" t="str">
+        <v>Day 1</v>
+      </c>
+      <c r="B4" s="10" t="str">
+        <v>10 June 2025</v>
+      </c>
+      <c r="C4" s="11" t="str">
+        <v>Uploaded</v>
+      </c>
+      <c r="D4" s="12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Small bruise forming on right upper arm. Alert and orientated. Reluctant to lift right arm above shoulder height.
+Immediate actions: Assisted to chair. Ice pack applied to shoulder. Call bell within reach.
+Vital signs: BP 162/94, HR 90, RR 17, Temp 36.7, SpO2 96%.
+GP (Dr Amir Nasseri) notified at 11:45. Advised X-ray of right shoulder to rule out fracture — to be arranged today. Resident transferred to radiology at 13:00, returned at 14:30. X-ray result pending.
+NOK: Daughter (Priya Singh) called at 12:00. Left voicemail — no response yet.
+Risk factors: Three falls in past year. Prescribed Apixaban — bleeding risk noted to GP. Bathroom grab rail present and in reach.
+Care plan: Will review tomorrow.</v>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1" xml:space="preserve">
+      <c r="A5" s="9" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B5" s="10" t="str">
+        <v>11 June 2025</v>
+      </c>
+      <c r="C5" s="11" t="str">
+        <v>Uploaded</v>
+      </c>
+      <c r="D5" s="12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+Mobilising carefully. Using left hand predominantly. Independent with walking.</v>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1" xml:space="preserve">
+      <c r="A6" s="9" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B6" s="10" t="str">
+        <v>12 June 2025</v>
+      </c>
+      <c r="C6" s="11" t="str">
+        <v>Uploaded</v>
+      </c>
+      <c r="D6" s="12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D16"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="4" max="4" width="90.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="4" t="str">
+        <v>Checker Output — Robert Singh</v>
+      </c>
+      <c r="B1" s="4" t="str">
+        <v/>
+      </c>
+      <c r="C1" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D1" s="4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="6" t="str">
+        <v>All 3 days reviewed against the Falls Management Policy.</v>
+      </c>
+      <c r="B2" s="6" t="str">
+        <v/>
+      </c>
+      <c r="C2" s="6" t="str">
+        <v/>
+      </c>
+      <c r="D2" s="6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="7" t="str">
+        <v>Day</v>
+      </c>
+      <c r="B3" s="7" t="str">
+        <v>Flag Type</v>
+      </c>
+      <c r="C3" s="7" t="str">
+        <v>Field</v>
+      </c>
+      <c r="D3" s="7" t="str">
+        <v>Explanation</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="str">
+        <v>Day 1</v>
+      </c>
+      <c r="B4" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C4" s="14" t="str">
+        <v>Witnessed status</v>
+      </c>
+      <c r="D4" s="14" t="str">
+        <v>Policy requires witnessed status to be documented. Note states 'Resident found on floor in bathroom', implying unwitnessed but policy requires explicit confirmation.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="str">
+        <v>Day 1</v>
+      </c>
+      <c r="B5" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C5" s="14" t="str">
+        <v>Falls risk score not reassessed</v>
+      </c>
+      <c r="D5" s="14" t="str">
+        <v>Policy requires a reassessed falls risk score. No falls risk score reassessment documented.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="str">
+        <v>Day 1</v>
+      </c>
+      <c r="B6" s="16" t="str">
+        <v>⚠️ Vague</v>
+      </c>
+      <c r="C6" s="16" t="str">
+        <v>Care plan update unconfirmed</v>
+      </c>
+      <c r="D6" s="16" t="str">
+        <v>Policy requires explicit care plan review confirmation. Note states 'Care plan: Will review tomorrow' but policy requires a Yes or No answer regarding review completion.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B7" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C7" s="14" t="str">
+        <v>Pain status not updated</v>
+      </c>
+      <c r="D7" s="14" t="str">
+        <v>Policy requires a numeric 0-10 pain score or description like 'pain resolved' with a number. Note states 'shoulder still sore but managing' but does not provide a numeric pain score.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B8" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C8" s="14" t="str">
+        <v>New symptoms not assessed</v>
+      </c>
+      <c r="D8" s="14" t="str">
+        <v>Policy requires explicit address of new symptoms since Day 1. No mention of new symptoms is made in the note.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B9" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C9" s="14" t="str">
+        <v>Vital signs not recorded</v>
+      </c>
+      <c r="D9" s="14" t="str">
+        <v>Policy requires a full set of vital signs. No vital signs are recorded in the note.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B10" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C10" s="14" t="str">
+        <v>Care plan changes not documented</v>
+      </c>
+      <c r="D10" s="14" t="str">
+        <v>Policy requires mention of care plan changes or explicit statement of no changes. The note does not address the care plan.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B11" s="16" t="str">
+        <v>⚠️ Vague</v>
+      </c>
+      <c r="C11" s="16" t="str">
+        <v>Mobility status unclear</v>
+      </c>
+      <c r="D11" s="16" t="str">
+        <v>Policy requires explicit statement on full weight-bearing status. Note states 'mobilising carefully' and 'independent with walking' but does not explicitly state whether the resident can full weight-bear without pain.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B12" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C12" s="14" t="str">
+        <v>Mobility not confirmed at baseline</v>
+      </c>
+      <c r="D12" s="14" t="str">
+        <v>Policy requires explicit confirmation of mobility status. No mobility status mentioned in the note.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B13" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C13" s="14" t="str">
+        <v>Outstanding actions not documented</v>
+      </c>
+      <c r="D13" s="14" t="str">
+        <v>Policy requires documentation of outstanding actions. No outstanding actions addressed in the note.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B14" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C14" s="14" t="str">
+        <v>Incident not formally closed</v>
+      </c>
+      <c r="D14" s="14" t="str">
+        <v>Policy requires formal incident closure statement. No incident closure statement found in the note.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B15" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C15" s="14" t="str">
+        <v>Falls prevention plan not reviewed</v>
+      </c>
+      <c r="D15" s="14" t="str">
+        <v>Policy requires review of falls prevention plan. No review or discussion of the falls prevention plan mentioned in the note.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B16" s="16" t="str">
+        <v>⚠️ Vague</v>
+      </c>
+      <c r="C16" s="16" t="str">
+        <v>Pain outcome not clinically confirmed</v>
+      </c>
+      <c r="D16" s="16" t="str">
+        <v>Policy requires clinically confirmed pain outcome. Note states 'Shoulder much better' but this is not a clinical confirmation of pain outcome.</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D16"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D6"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="90.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="4" t="str">
+        <v>Progress Notes — Thomas Brennan</v>
+      </c>
+      <c r="B1" s="4" t="str">
+        <v/>
+      </c>
+      <c r="C1" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D1" s="4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="6" t="str">
+        <v>3 consecutive daily progress notes uploaded for compliance checking.</v>
+      </c>
+      <c r="B2" s="6" t="str">
+        <v/>
+      </c>
+      <c r="C2" s="6" t="str">
+        <v/>
+      </c>
+      <c r="D2" s="6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="8" t="str">
+        <v>Day</v>
+      </c>
+      <c r="B3" s="8" t="str">
+        <v>Date</v>
+      </c>
+      <c r="C3" s="8" t="str">
+        <v>Source</v>
+      </c>
+      <c r="D3" s="8" t="str">
+        <v>Progress Note</v>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1" xml:space="preserve">
+      <c r="A4" s="9" t="str">
+        <v>Day 1</v>
+      </c>
+      <c r="B4" s="10" t="str">
+        <v>10 June 2025</v>
+      </c>
+      <c r="C4" s="11" t="str">
+        <v>Uploaded</v>
+      </c>
+      <c r="D4" s="12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Progress Note — Fall Incident
+Resident: Thomas Brennan  |  Room: 9F  |  DOB: 22/05/1941
+Date: 10 June 2025  |  Time of fall: 13:55
+Resident witnessed falling in the activity room. Complaining of left knee pain — rates 5/10. No visible injury. Alert and orientated. Able to move all limbs.
+Immediate actions: Assisted to chair. Comfort measures applied. Call bell within reach.
+Vital signs: BP 145/88, HR 82, RR 16, Temp 36.6, SpO2 97%.
+GP (Dr Maria Santos) notified at 14:15. Advised to monitor and reassess tomorrow.
+NOK: Wife (Catherine Brennan) notified at 14:30. Acknowledged, will visit this evening.
+Risk factors: Two previous falls this year. On Warfarin — bleeding risk noted. Uses walking stick.
+Walking stick was in reach at time of fall.
+Care plan reviewed and updated: Yes. Walking stick protocol reinforced. Falls risk score reassessed — HIGH.</v>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1" xml:space="preserve">
+      <c r="A5" s="9" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B5" s="10" t="str">
+        <v>11 June 2025</v>
+      </c>
+      <c r="C5" s="11" t="str">
+        <v>Uploaded</v>
+      </c>
+      <c r="D5" s="12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, HR 78, RR 15, Temp 36.5, SpO2 98%.
+GP contacted at 10:00 — Dr Santos updated on improvement. No further action required at this stage. Wife visited last night.</v>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1" xml:space="preserve">
+      <c r="A6" s="9" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B6" s="10" t="str">
+        <v>12 June 2025</v>
+      </c>
+      <c r="C6" s="11" t="str">
+        <v>Uploaded</v>
+      </c>
+      <c r="D6" s="12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this afternoon.</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D10"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="4" max="4" width="90.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="4" t="str">
+        <v>Checker Output — Thomas Brennan</v>
+      </c>
+      <c r="B1" s="4" t="str">
+        <v/>
+      </c>
+      <c r="C1" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D1" s="4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="6" t="str">
+        <v>All 3 days reviewed against the Falls Management Policy.</v>
+      </c>
+      <c r="B2" s="6" t="str">
+        <v/>
+      </c>
+      <c r="C2" s="6" t="str">
+        <v/>
+      </c>
+      <c r="D2" s="6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="7" t="str">
+        <v>Day</v>
+      </c>
+      <c r="B3" s="7" t="str">
+        <v>Flag Type</v>
+      </c>
+      <c r="C3" s="7" t="str">
+        <v>Field</v>
+      </c>
+      <c r="D3" s="7" t="str">
+        <v>Explanation</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="str">
+        <v>Day 1</v>
+      </c>
+      <c r="B4" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C4" s="14" t="str">
+        <v>GP conditional actions not documented</v>
+      </c>
+      <c r="D4" s="14" t="str">
+        <v>Policy requires GP advice to include specific conditional actions with clear thresholds or triggers. Note states 'advised to monitor and reassess tomorrow,' which is generic monitoring advice without specific triggers or thresholds.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B5" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C5" s="14" t="str">
+        <v>New symptoms not assessed</v>
+      </c>
+      <c r="D5" s="14" t="str">
+        <v>Policy requires explicit documentation of whether there are any new symptoms since Day 1. The note does not address this question, and no mention of new or absent symptoms is made.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B6" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C6" s="14" t="str">
+        <v>Care plan changes not documented</v>
+      </c>
+      <c r="D6" s="14" t="str">
+        <v>Policy requires documentation of care plan changes or a statement that there are no changes. The note does not mention the care plan at all.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B7" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C7" s="14" t="str">
+        <v>Outstanding actions not documented</v>
+      </c>
+      <c r="D7" s="14" t="str">
+        <v>Policy requires documentation of whether prior actions have been resolved. No mention of outstanding actions from previous days is included in the note.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B8" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C8" s="14" t="str">
+        <v>Incident not formally closed</v>
+      </c>
+      <c r="D8" s="14" t="str">
+        <v>Policy requires a formal statement that the post-fall monitoring period is complete and the incident is closed. No such statement is present in the note.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B9" s="14" t="str">
+        <v>🚩 Missing</v>
+      </c>
+      <c r="C9" s="14" t="str">
+        <v>Falls prevention plan not reviewed</v>
+      </c>
+      <c r="D9" s="14" t="str">
+        <v>Policy requires confirmation that the updated falls prevention plan was reviewed or discussed with the resident and/or family. No mention of a falls prevention plan review or discussion is included in the note.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B10" s="16" t="str">
+        <v>⚠️ Vague</v>
+      </c>
+      <c r="C10" s="16" t="str">
+        <v>Mobility not confirmed at baseline</v>
+      </c>
+      <c r="D10" s="16" t="str">
+        <v>Policy requires explicit confirmation of mobility status as returned to baseline or reduced with a follow-up plan. Note states 'mobilising independently with walking stick, no concerns,' but does not confirm if this is baseline mobility.</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>